<commit_message>
Weekly GA4 tables update 2026-09-14
</commit_message>
<xml_diff>
--- a/exports/Seeed周度三表_W23-W36_2026-09-13.xlsx
+++ b/exports/Seeed周度三表_W23-W36_2026-09-13.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="方案增长总览" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="单方案流量明细" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="转换漏斗" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="方案增长总览" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="单方案流量明细" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="转换漏斗" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -515,19 +515,19 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>548</v>
+        <v>782</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>561</v>
+        <v>897</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>8.199999999999999</v>
+        <v>6.91</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-50.9</v>
+        <v>-21.5</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -536,7 +536,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>室内外定位 (+-13.6%)</t>
+          <t>室内外定位 (+27.3%)</t>
         </is>
       </c>
     </row>
@@ -1007,50 +1007,13 @@
       <c r="F15" s="2" t="n">
         <v>12.66</v>
       </c>
-      <c r="G15" s="2" t="n">
-        <v>-6.4</v>
-      </c>
+      <c r="G15" s="2" t="n"/>
       <c r="H15" s="2" t="inlineStr">
         <is>
           <t>对话式语音AI</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>智能视频分析 (+27.3%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>614</v>
-      </c>
-      <c r="D16" s="2" t="n">
-        <v>751</v>
-      </c>
-      <c r="E16" s="2" t="n">
-        <v>77</v>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>10.25</v>
-      </c>
-      <c r="G16" s="2" t="n"/>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>对话式语音AI</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1063,7 +1026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M181"/>
+  <dimension ref="A1:M169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1165,19 +1128,19 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>117</v>
+        <v>178</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>114</v>
+        <v>165</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>127</v>
+        <v>183</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>21.2</v>
+        <v>24.1</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>29.13</v>
+        <v>41.53</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -1185,13 +1148,13 @@
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>-40.6</v>
+        <v>-9.6</v>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
@@ -1216,19 +1179,19 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>103</v>
+        <v>162</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>100</v>
+        <v>144</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>121</v>
+        <v>174</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>62.8</v>
+        <v>57.6</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>52.89</v>
+        <v>65.52</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -1236,13 +1199,13 @@
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>-50.5</v>
+        <v>-22.1</v>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
@@ -1267,19 +1230,19 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>61</v>
+        <v>90</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>18.9</v>
+        <v>33.6</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>42.62</v>
+        <v>58.89</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -1287,13 +1250,13 @@
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="K4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>-46.4</v>
+        <v>-10.7</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
@@ -1314,23 +1277,23 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>智能仓储管理</t>
+          <t>智慧畜牧</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>58</v>
+        <v>83</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>41.2</v>
+        <v>13.6</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46.55</v>
+        <v>55.42</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -1338,13 +1301,13 @@
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>-47.7</v>
+        <v>-28</v>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
@@ -1365,23 +1328,23 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>智慧畜牧</t>
+          <t>智能视频分析</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>8.6</v>
+        <v>78.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>50</v>
+        <v>61.19</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
@@ -1389,13 +1352,13 @@
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>-62.7</v>
+        <v>-46.6</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
@@ -1416,37 +1379,37 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>智能视频分析</t>
+          <t>智能仓储管理</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>38</v>
+        <v>68</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>70.09999999999999</v>
+        <v>37.3</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>47.73</v>
+        <v>67.11</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Unassigned</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="J7" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>-71.40000000000001</v>
+        <v>-20.9</v>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
@@ -1471,19 +1434,19 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>27.6</v>
+        <v>29</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1491,13 +1454,13 @@
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>-13.6</v>
+        <v>27.3</v>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
@@ -1518,23 +1481,23 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>校园安全管理</t>
+          <t>环境监测</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>31</v>
+        <v>54</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>21.4</v>
+        <v>48.4</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>42.11</v>
+        <v>67.27</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1542,13 +1505,13 @@
         </is>
       </c>
       <c r="J9" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>-20.5</v>
+        <v>-16.9</v>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
@@ -1573,19 +1536,19 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>29.5</v>
+        <v>32.1</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>60</v>
+        <v>67.39</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1599,7 +1562,7 @@
         <v>0</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>-40</v>
+        <v>-14</v>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
@@ -1620,23 +1583,23 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>环境监测</t>
+          <t>校园安全管理</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>33.8</v>
+        <v>22.8</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>51.61</v>
+        <v>66.67</v>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
@@ -1644,13 +1607,13 @@
         </is>
       </c>
       <c r="J11" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>-56.9</v>
+        <v>5.1</v>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
@@ -1675,19 +1638,19 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>33.1</v>
+        <v>29.5</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>66.67</v>
+        <v>78.26000000000001</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
@@ -1701,7 +1664,7 @@
         <v>0</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>-66.7</v>
+        <v>-51.1</v>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
@@ -1726,19 +1689,19 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>76.40000000000001</v>
+        <v>66.2</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>62.5</v>
+        <v>78.95</v>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
@@ -1752,7 +1715,7 @@
         <v>0</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>-73.90000000000001</v>
+        <v>-63</v>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
@@ -9146,9 +9109,7 @@
       <c r="K158" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="L158" s="2" t="n">
-        <v>-4.2</v>
-      </c>
+      <c r="L158" s="2" t="n"/>
       <c r="M158" s="2" t="inlineStr">
         <is>
           <t>GA4+LeadApi已接入</t>
@@ -9197,9 +9158,7 @@
       <c r="K159" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L159" s="2" t="n">
-        <v>5.6</v>
-      </c>
+      <c r="L159" s="2" t="n"/>
       <c r="M159" s="2" t="inlineStr">
         <is>
           <t>GA4+LeadApi已接入</t>
@@ -9248,9 +9207,7 @@
       <c r="K160" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L160" s="2" t="n">
-        <v>-10.7</v>
-      </c>
+      <c r="L160" s="2" t="n"/>
       <c r="M160" s="2" t="inlineStr">
         <is>
           <t>GA4+LeadApi已接入</t>
@@ -9299,9 +9256,7 @@
       <c r="K161" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L161" s="2" t="n">
-        <v>12</v>
-      </c>
+      <c r="L161" s="2" t="n"/>
       <c r="M161" s="2" t="inlineStr">
         <is>
           <t>GA4+LeadApi已接入</t>
@@ -9350,9 +9305,7 @@
       <c r="K162" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L162" s="2" t="n">
-        <v>27.3</v>
-      </c>
+      <c r="L162" s="2" t="n"/>
       <c r="M162" s="2" t="inlineStr">
         <is>
           <t>GA4+LeadApi已接入</t>
@@ -9401,9 +9354,7 @@
       <c r="K163" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L163" s="2" t="n">
-        <v>1.9</v>
-      </c>
+      <c r="L163" s="2" t="n"/>
       <c r="M163" s="2" t="inlineStr">
         <is>
           <t>GA4+LeadApi已接入</t>
@@ -9452,9 +9403,7 @@
       <c r="K164" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L164" s="2" t="n">
-        <v>-15.3</v>
-      </c>
+      <c r="L164" s="2" t="n"/>
       <c r="M164" s="2" t="inlineStr">
         <is>
           <t>GA4+LeadApi已接入</t>
@@ -9503,9 +9452,7 @@
       <c r="K165" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L165" s="2" t="n">
-        <v>-25.4</v>
-      </c>
+      <c r="L165" s="2" t="n"/>
       <c r="M165" s="2" t="inlineStr">
         <is>
           <t>GA4+LeadApi已接入</t>
@@ -9554,9 +9501,7 @@
       <c r="K166" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L166" s="2" t="n">
-        <v>-35.5</v>
-      </c>
+      <c r="L166" s="2" t="n"/>
       <c r="M166" s="2" t="inlineStr">
         <is>
           <t>GA4+LeadApi已接入</t>
@@ -9605,9 +9550,7 @@
       <c r="K167" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L167" s="2" t="n">
-        <v>-2.9</v>
-      </c>
+      <c r="L167" s="2" t="n"/>
       <c r="M167" s="2" t="inlineStr">
         <is>
           <t>GA4+LeadApi已接入</t>
@@ -9656,9 +9599,7 @@
       <c r="K168" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L168" s="2" t="n">
-        <v>6.5</v>
-      </c>
+      <c r="L168" s="2" t="n"/>
       <c r="M168" s="2" t="inlineStr">
         <is>
           <t>GA4+LeadApi已接入</t>
@@ -9707,598 +9648,8 @@
       <c r="K169" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L169" s="2" t="n">
-        <v>-29.5</v>
-      </c>
+      <c r="L169" s="2" t="n"/>
       <c r="M169" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B170" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C170" s="2" t="inlineStr">
-        <is>
-          <t>对话式语音AI</t>
-        </is>
-      </c>
-      <c r="D170" s="2" t="n">
-        <v>119</v>
-      </c>
-      <c r="E170" s="2" t="n">
-        <v>94</v>
-      </c>
-      <c r="F170" s="2" t="n">
-        <v>125</v>
-      </c>
-      <c r="G170" s="2" t="n">
-        <v>51.1</v>
-      </c>
-      <c r="H170" s="2" t="n">
-        <v>73.59999999999999</v>
-      </c>
-      <c r="I170" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="J170" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="K170" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L170" s="2" t="n"/>
-      <c r="M170" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B171" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C171" s="2" t="inlineStr">
-        <is>
-          <t>语音采集分析</t>
-        </is>
-      </c>
-      <c r="D171" s="2" t="n">
-        <v>107</v>
-      </c>
-      <c r="E171" s="2" t="n">
-        <v>85</v>
-      </c>
-      <c r="F171" s="2" t="n">
-        <v>104</v>
-      </c>
-      <c r="G171" s="2" t="n">
-        <v>37.4</v>
-      </c>
-      <c r="H171" s="2" t="n">
-        <v>69.23</v>
-      </c>
-      <c r="I171" s="2" t="inlineStr">
-        <is>
-          <t>Referral</t>
-        </is>
-      </c>
-      <c r="J171" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="K171" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L171" s="2" t="n"/>
-      <c r="M171" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B172" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C172" s="2" t="inlineStr">
-        <is>
-          <t>智慧农业感知</t>
-        </is>
-      </c>
-      <c r="D172" s="2" t="n">
-        <v>84</v>
-      </c>
-      <c r="E172" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="F172" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="G172" s="2" t="n">
-        <v>38.6</v>
-      </c>
-      <c r="H172" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="I172" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="J172" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K172" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L172" s="2" t="n"/>
-      <c r="M172" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B173" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C173" s="2" t="inlineStr">
-        <is>
-          <t>楼宇节能改造</t>
-        </is>
-      </c>
-      <c r="D173" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="E173" s="2" t="n">
-        <v>47</v>
-      </c>
-      <c r="F173" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="G173" s="2" t="n">
-        <v>31.1</v>
-      </c>
-      <c r="H173" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="I173" s="2" t="inlineStr">
-        <is>
-          <t>Referral</t>
-        </is>
-      </c>
-      <c r="J173" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="K173" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L173" s="2" t="n"/>
-      <c r="M173" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B174" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C174" s="2" t="inlineStr">
-        <is>
-          <t>室内外定位</t>
-        </is>
-      </c>
-      <c r="D174" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="E174" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="F174" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="G174" s="2" t="n">
-        <v>49.3</v>
-      </c>
-      <c r="H174" s="2" t="n">
-        <v>78.69</v>
-      </c>
-      <c r="I174" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="J174" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K174" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L174" s="2" t="n"/>
-      <c r="M174" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B175" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C175" s="2" t="inlineStr">
-        <is>
-          <t>环境监测</t>
-        </is>
-      </c>
-      <c r="D175" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="E175" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="F175" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="G175" s="2" t="n">
-        <v>37.1</v>
-      </c>
-      <c r="H175" s="2" t="n">
-        <v>77.78</v>
-      </c>
-      <c r="I175" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="J175" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="K175" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L175" s="2" t="n"/>
-      <c r="M175" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B176" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C176" s="2" t="inlineStr">
-        <is>
-          <t>智能仓储管理</t>
-        </is>
-      </c>
-      <c r="D176" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="E176" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="F176" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="G176" s="2" t="n">
-        <v>27.8</v>
-      </c>
-      <c r="H176" s="2" t="n">
-        <v>84.44</v>
-      </c>
-      <c r="I176" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="J176" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K176" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L176" s="2" t="n"/>
-      <c r="M176" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B177" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C177" s="2" t="inlineStr">
-        <is>
-          <t>智慧畜牧</t>
-        </is>
-      </c>
-      <c r="D177" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="E177" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="F177" s="2" t="n">
-        <v>43</v>
-      </c>
-      <c r="G177" s="2" t="n">
-        <v>34.6</v>
-      </c>
-      <c r="H177" s="2" t="n">
-        <v>76.73999999999999</v>
-      </c>
-      <c r="I177" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="J177" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="K177" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L177" s="2" t="n"/>
-      <c r="M177" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B178" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C178" s="2" t="inlineStr">
-        <is>
-          <t>智能视频分析</t>
-        </is>
-      </c>
-      <c r="D178" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="E178" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="F178" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="G178" s="2" t="n">
-        <v>45.7</v>
-      </c>
-      <c r="H178" s="2" t="n">
-        <v>61.22</v>
-      </c>
-      <c r="I178" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="J178" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="K178" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L178" s="2" t="n"/>
-      <c r="M178" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B179" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C179" s="2" t="inlineStr">
-        <is>
-          <t>楼宇能源管理</t>
-        </is>
-      </c>
-      <c r="D179" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="E179" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="F179" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="G179" s="2" t="n">
-        <v>47.4</v>
-      </c>
-      <c r="H179" s="2" t="n">
-        <v>77.55</v>
-      </c>
-      <c r="I179" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="J179" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K179" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L179" s="2" t="n"/>
-      <c r="M179" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B180" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C180" s="2" t="inlineStr">
-        <is>
-          <t>应急响应</t>
-        </is>
-      </c>
-      <c r="D180" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="E180" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="F180" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="G180" s="2" t="n">
-        <v>28.7</v>
-      </c>
-      <c r="H180" s="2" t="n">
-        <v>74.29000000000001</v>
-      </c>
-      <c r="I180" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="J180" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K180" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L180" s="2" t="n"/>
-      <c r="M180" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B181" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C181" s="2" t="inlineStr">
-        <is>
-          <t>校园安全管理</t>
-        </is>
-      </c>
-      <c r="D181" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="E181" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="F181" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="G181" s="2" t="n">
-        <v>37.7</v>
-      </c>
-      <c r="H181" s="2" t="n">
-        <v>81.81999999999999</v>
-      </c>
-      <c r="I181" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="J181" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K181" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L181" s="2" t="n"/>
-      <c r="M181" s="2" t="inlineStr">
         <is>
           <t>GA4+LeadApi已接入</t>
         </is>
@@ -10315,7 +9666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J181"/>
+  <dimension ref="A1:J169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10399,19 +9750,19 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>117</v>
+        <v>178</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>127</v>
+        <v>183</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>2.56</v>
+        <v>3.37</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>0</v>
@@ -10439,22 +9790,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>103</v>
+        <v>162</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>121</v>
+        <v>174</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>12.62</v>
+        <v>9.26</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>0.97</v>
+        <v>0.62</v>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
@@ -10479,19 +9830,19 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>61</v>
+        <v>90</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>0</v>
@@ -10515,23 +9866,23 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>智能仓储管理</t>
+          <t>智慧畜牧</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>58</v>
+        <v>83</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>11.11</v>
+        <v>3.53</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>0</v>
@@ -10555,23 +9906,23 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>智慧畜牧</t>
+          <t>智能视频分析</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>0</v>
@@ -10595,23 +9946,23 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>智能视频分析</t>
+          <t>智能仓储管理</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>38</v>
+        <v>68</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>18.42</v>
+        <v>8.82</v>
       </c>
       <c r="I7" s="2" t="n">
         <v>0</v>
@@ -10639,19 +9990,19 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>13.16</v>
+        <v>10.71</v>
       </c>
       <c r="I8" s="2" t="n">
         <v>0</v>
@@ -10675,23 +10026,23 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>校园安全管理</t>
+          <t>环境监测</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>31</v>
+        <v>54</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>3.23</v>
+        <v>0</v>
       </c>
       <c r="I9" s="2" t="n">
         <v>0</v>
@@ -10719,10 +10070,10 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>0</v>
@@ -10755,23 +10106,23 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>环境监测</t>
+          <t>校园安全管理</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>0</v>
+        <v>7.32</v>
       </c>
       <c r="I11" s="2" t="n">
         <v>0</v>
@@ -10799,10 +10150,10 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F12" s="2" t="n">
         <v>0</v>
@@ -10839,10 +10190,10 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F13" s="2" t="n">
         <v>3</v>
@@ -10851,7 +10202,7 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>25</v>
+        <v>17.65</v>
       </c>
       <c r="I13" s="2" t="n">
         <v>0</v>
@@ -17097,486 +16448,6 @@
         <v>0</v>
       </c>
       <c r="J169" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B170" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C170" s="2" t="inlineStr">
-        <is>
-          <t>对话式语音AI</t>
-        </is>
-      </c>
-      <c r="D170" s="2" t="n">
-        <v>119</v>
-      </c>
-      <c r="E170" s="2" t="n">
-        <v>125</v>
-      </c>
-      <c r="F170" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="G170" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H170" s="2" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="I170" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J170" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B171" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C171" s="2" t="inlineStr">
-        <is>
-          <t>语音采集分析</t>
-        </is>
-      </c>
-      <c r="D171" s="2" t="n">
-        <v>107</v>
-      </c>
-      <c r="E171" s="2" t="n">
-        <v>104</v>
-      </c>
-      <c r="F171" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="G171" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H171" s="2" t="n">
-        <v>14.95</v>
-      </c>
-      <c r="I171" s="2" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="J171" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B172" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C172" s="2" t="inlineStr">
-        <is>
-          <t>智慧农业感知</t>
-        </is>
-      </c>
-      <c r="D172" s="2" t="n">
-        <v>84</v>
-      </c>
-      <c r="E172" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="F172" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="G172" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H172" s="2" t="n">
-        <v>5.95</v>
-      </c>
-      <c r="I172" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J172" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B173" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C173" s="2" t="inlineStr">
-        <is>
-          <t>楼宇节能改造</t>
-        </is>
-      </c>
-      <c r="D173" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="E173" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="F173" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="G173" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H173" s="2" t="n">
-        <v>28.57</v>
-      </c>
-      <c r="I173" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J173" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B174" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C174" s="2" t="inlineStr">
-        <is>
-          <t>室内外定位</t>
-        </is>
-      </c>
-      <c r="D174" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="E174" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="F174" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G174" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H174" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I174" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J174" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B175" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C175" s="2" t="inlineStr">
-        <is>
-          <t>环境监测</t>
-        </is>
-      </c>
-      <c r="D175" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="E175" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="F175" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="G175" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H175" s="2" t="n">
-        <v>15.25</v>
-      </c>
-      <c r="I175" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J175" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B176" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C176" s="2" t="inlineStr">
-        <is>
-          <t>智能仓储管理</t>
-        </is>
-      </c>
-      <c r="D176" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="E176" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="F176" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G176" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H176" s="2" t="n">
-        <v>3.77</v>
-      </c>
-      <c r="I176" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J176" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B177" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C177" s="2" t="inlineStr">
-        <is>
-          <t>智慧畜牧</t>
-        </is>
-      </c>
-      <c r="D177" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="E177" s="2" t="n">
-        <v>43</v>
-      </c>
-      <c r="F177" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G177" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H177" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="I177" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J177" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B178" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C178" s="2" t="inlineStr">
-        <is>
-          <t>智能视频分析</t>
-        </is>
-      </c>
-      <c r="D178" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="E178" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="F178" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="G178" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H178" s="2" t="n">
-        <v>20.45</v>
-      </c>
-      <c r="I178" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J178" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B179" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C179" s="2" t="inlineStr">
-        <is>
-          <t>楼宇能源管理</t>
-        </is>
-      </c>
-      <c r="D179" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="E179" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="F179" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G179" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H179" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I179" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J179" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B180" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C180" s="2" t="inlineStr">
-        <is>
-          <t>应急响应</t>
-        </is>
-      </c>
-      <c r="D180" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="E180" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="F180" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G180" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H180" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I180" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J180" s="2" t="inlineStr">
-        <is>
-          <t>GA4+LeadApi已接入</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" s="2" t="inlineStr">
-        <is>
-          <t>W23</t>
-        </is>
-      </c>
-      <c r="B181" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C181" s="2" t="inlineStr">
-        <is>
-          <t>校园安全管理</t>
-        </is>
-      </c>
-      <c r="D181" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="E181" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="F181" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="G181" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H181" s="2" t="n">
-        <v>16.13</v>
-      </c>
-      <c r="I181" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J181" s="2" t="inlineStr">
         <is>
           <t>GA4+LeadApi已接入</t>
         </is>

</xml_diff>